<commit_message>
Backup current project state
</commit_message>
<xml_diff>
--- a/Wikidata Delta/om_gen_excels/pep_oman_living_relevant_rca_lookup.xlsx
+++ b/Wikidata Delta/om_gen_excels/pep_oman_living_relevant_rca_lookup.xlsx
@@ -443,180 +443,180 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Awad bin Arfah bin Frijoon Bait Sameer</t>
+          <t>Sanaa Al Haib</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>OM-GEN-ABABFBS-Y5L23-RCA-1</t>
+          <t>OM-GEN-SAH-I7QQH-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bilarab bin Haitham Al Said</t>
+          <t>Ahad bint Abdullah Al Busaidi</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OM-GEN-BBHAS-K1GPH-RCA-1</t>
+          <t>OM-GEN-ABAAB-W4WCP-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Theyazin bin Haitham Al Said</t>
+          <t>Awad bin Arfah bin Frijoon Bait Sameer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OM-GEN-TBHAS-4JERL-RCA-1</t>
+          <t>OM-GEN-ABABFBS-SRX09-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mai Almasri</t>
+          <t>Bilarab bin Haitham Al Said</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OM-GEN-MA-LVP7J-RCA-1</t>
+          <t>OM-GEN-BBHAS-W9Z5Y-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Taimur bin Asaad Al Said</t>
+          <t>Theyazin bin Haitham Al Said</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>OM-GEN-TBAAS-ADW8S-RCA-1</t>
+          <t>OM-GEN-TBHAS-HR39A-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Meyyan bint Shihab Al Said</t>
+          <t>Mai Almasri</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OM-GEN-MBSAS-2Q18K-RCA-1</t>
+          <t>OM-GEN-MA-9FJMS-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Shawana bint Hammoud Al Busaidi</t>
+          <t>Taimur bin Asaad Al Said</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>OM-GEN-SBHAB-31X4Q-RCA-1</t>
+          <t>OM-GEN-TBAAS-07PX3-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Asa ad bin Tariq Al Said</t>
+          <t>Meyyan bint Shihab Al Said</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>OM-GEN-AABTAS-N0PVG-RCA-1</t>
+          <t>OM-GEN-MBSAS-JDDM5-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nawwal bint Tariq Al Said</t>
+          <t>Shawana bint Hammoud Al Busaidi</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>OM-GEN-NBTAS-D267A-RCA-1</t>
+          <t>OM-GEN-SBHAB-SSFCD-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shihab bin Tariq Al Said</t>
+          <t>Asa ad bin Tariq Al Said</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>OM-GEN-SBTAS-TZ8KW-RCA-1</t>
+          <t>OM-GEN-AABTAS-PHK8T-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Badr bin Hamad Al Busaidi</t>
+          <t>Nawwal bint Tariq Al Said</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>OM-GEN-BBHAB-O66NC-RCA-1</t>
+          <t>OM-GEN-NBTAS-SR4YA-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Haitham bin Tarik Al Said</t>
+          <t>Shihab bin Tariq Al Said</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>OM-GEN-HBTAS-NFVFQ-RCA-1</t>
+          <t>OM-GEN-SBTAS-H1WT0-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Khalid bin Hilal Al Busaidi</t>
+          <t>Badr bin Hamad Al Busaidi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>OM-GEN-KBHAB-VTYKP-RCA-1</t>
+          <t>OM-GEN-BBHAB-4HR4W-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sanaa Al Haib</t>
+          <t>Haitham bin Tarik Al Said</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>OM-GEN-SAH-TE5LH-RCA-1</t>
+          <t>OM-GEN-HBTAS-8RB04-RCA-1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ahad bint Abdullah Al Busaidi</t>
+          <t>Khalid bin Hilal Al Busaidi</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OM-GEN-ABAAB-F7B1T-RCA-1</t>
+          <t>OM-GEN-KBHAB-O1ZEC-RCA-1</t>
         </is>
       </c>
     </row>

</xml_diff>